<commit_message>
Day 2 of my journey to keep on growing starting with excel to strengthen the base and gaining the mindset
</commit_message>
<xml_diff>
--- a/Working/Excel Working/04122025_Winter_Fashion_Trends/Winter_Fashion_Trends_Dataset.xlsx
+++ b/Working/Excel Working/04122025_Winter_Fashion_Trends/Winter_Fashion_Trends_Dataset.xlsx
@@ -8,16 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sahil\OneDrive\Documents\Git_Repositories\Daily-Concept-Proofing\Working\Excel Working\04122025_Winter_Fashion_Trends\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{2E1C5CFF-7B00-4892-AE2D-34C890A2AE0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6F48B6-E55F-45E9-9D5F-8DE8ABF92BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{4AEEEB2B-2F7C-4B17-B97E-AA8A0F82D82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Winter_Fashion_Trends_DS(OG)" sheetId="1" r:id="rId1"/>
     <sheet name="Analyzing_DS" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Analyzing_DS!$A$1:$L$151</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -44,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2439" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2463" uniqueCount="74">
   <si>
     <t>ID</t>
   </si>
@@ -250,6 +263,24 @@
   </si>
   <si>
     <t>Rank Based on Popularity</t>
+  </si>
+  <si>
+    <t>Materials</t>
+  </si>
+  <si>
+    <t>Market Median Price</t>
+  </si>
+  <si>
+    <t>Market Price for Uniqlo</t>
+  </si>
+  <si>
+    <t>%Differcnce between Uniqolo and Market</t>
+  </si>
+  <si>
+    <t>Count of Woolean Item sold by Uniqlo</t>
+  </si>
+  <si>
+    <t>Price of the Product</t>
   </si>
 </sst>
 </file>
@@ -770,7 +801,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -816,21 +849,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -856,10 +875,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6921,7 +6936,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F49F8F5A-4B24-4E07-AC3A-C9E0A622917F}">
-  <dimension ref="A1:T151"/>
+  <dimension ref="A1:Y151"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -6936,12 +6951,18 @@
     <col min="10" max="10" width="15.44140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="18" width="10" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.21875" customWidth="1"/>
+    <col min="18" max="18" width="18.33203125" customWidth="1"/>
     <col min="19" max="19" width="10.21875" customWidth="1"/>
     <col min="20" max="20" width="10.5546875" customWidth="1"/>
+    <col min="22" max="22" width="11.33203125" customWidth="1"/>
+    <col min="23" max="23" width="13" customWidth="1"/>
+    <col min="24" max="24" width="14.33203125" customWidth="1"/>
+    <col min="25" max="25" width="15.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="4" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:25" s="4" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -6993,8 +7014,20 @@
       <c r="T1" s="5" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="V1" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="W1" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="X1" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="Y1" s="7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -7043,15 +7076,30 @@
         <v>468.58</v>
       </c>
       <c r="S2" s="6">
-        <f>AVERAGEIFS($J$2:$J$151,$B$2:$B$151,P2)</f>
+        <f t="shared" ref="S2:S11" si="0">AVERAGEIFS($J$2:$J$151,$B$2:$B$151,P2)</f>
         <v>6.5279999999999996</v>
       </c>
-      <c r="T2" s="7">
-        <f>_xlfn.RANK.AVG(S2,$S$2:$S$11,0)</f>
+      <c r="T2" s="1">
+        <f t="shared" ref="T2:T11" si="1">_xlfn.RANK.AVG(S2,$S$2:$S$11,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="V2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W2" s="1" cm="1">
+        <f t="array" ref="W2">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,0,$E$2:$E$151=$V2),0))</f>
+        <v>344.54499999999996</v>
+      </c>
+      <c r="X2" s="1">
+        <f t="array" ref="X2">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,$E$2:$E$151=$V2,0),0))</f>
+        <v>677.98</v>
+      </c>
+      <c r="Y2" s="6" cm="1">
+        <f t="array" ref="Y2">IFERROR((X2/W2)*100,NA)</f>
+        <v>196.77545748741096</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -7100,15 +7148,30 @@
         <v>399.37</v>
       </c>
       <c r="S3" s="6">
-        <f>AVERAGEIFS($J$2:$J$151,$B$2:$B$151,P3)</f>
+        <f t="shared" si="0"/>
         <v>6.4846153846153847</v>
       </c>
-      <c r="T3" s="7">
-        <f>_xlfn.RANK.AVG(S3,$S$2:$S$11,0)</f>
+      <c r="T3" s="1">
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="V3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="W3" s="1" cm="1">
+        <f t="array" ref="W3">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,0,$E$2:$E$151=$V3),0))</f>
+        <v>437.69</v>
+      </c>
+      <c r="X3" s="1">
+        <f t="array" ref="X3">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,$E$2:$E$151=$V3,0),0))</f>
+        <v>738.25</v>
+      </c>
+      <c r="Y3" s="6" cm="1">
+        <f t="array" ref="Y3">IFERROR((X3/W3)*100,NA)</f>
+        <v>168.66960634238845</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -7157,15 +7220,30 @@
         <v>367.56</v>
       </c>
       <c r="S4" s="6">
-        <f>AVERAGEIFS($J$2:$J$151,$B$2:$B$151,P4)</f>
+        <f t="shared" si="0"/>
         <v>6.4615384615384617</v>
       </c>
-      <c r="T4" s="7">
-        <f>_xlfn.RANK.AVG(S4,$S$2:$S$11,0)</f>
+      <c r="T4" s="1">
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="V4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="W4" s="1" cm="1">
+        <f t="array" ref="W4">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,0,$E$2:$E$151=$V4),0))</f>
+        <v>536.20000000000005</v>
+      </c>
+      <c r="X4" s="1">
+        <f t="array" ref="X4">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,$E$2:$E$151=$V4,0),0))</f>
+        <v>644.97</v>
+      </c>
+      <c r="Y4" s="6" cm="1">
+        <f t="array" ref="Y4">IFERROR((X4/W4)*100,NA)</f>
+        <v>120.28534129056321</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -7214,15 +7292,30 @@
         <v>555.62</v>
       </c>
       <c r="S5" s="6">
-        <f>AVERAGEIFS($J$2:$J$151,$B$2:$B$151,P5)</f>
+        <f t="shared" si="0"/>
         <v>6.2700000000000005</v>
       </c>
-      <c r="T5" s="7">
-        <f>_xlfn.RANK.AVG(S5,$S$2:$S$11,0)</f>
+      <c r="T5" s="1">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="V5" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="W5" s="1" cm="1">
+        <f t="array" ref="W5">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,0,$E$2:$E$151=$V5),0))</f>
+        <v>559.9</v>
+      </c>
+      <c r="X5" s="1">
+        <f t="array" ref="X5">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,$E$2:$E$151=$V5,0),0))</f>
+        <v>618.52499999999998</v>
+      </c>
+      <c r="Y5" s="6" cm="1">
+        <f t="array" ref="Y5">IFERROR((X5/W5)*100,NA)</f>
+        <v>110.47061975352742</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -7271,15 +7364,30 @@
         <v>358.65</v>
       </c>
       <c r="S6" s="6">
-        <f>AVERAGEIFS($J$2:$J$151,$B$2:$B$151,P6)</f>
+        <f t="shared" si="0"/>
         <v>5.8549999999999995</v>
       </c>
-      <c r="T6" s="7">
-        <f>_xlfn.RANK.AVG(S6,$S$2:$S$11,0)</f>
+      <c r="T6" s="1">
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="V6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="1" cm="1">
+        <f t="array" ref="W6">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,0,$E$2:$E$151=$V6),0))</f>
+        <v>445.18</v>
+      </c>
+      <c r="X6" s="1">
+        <f t="array" ref="X6">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,$E$2:$E$151=$V6,0),0))</f>
+        <v>439.44500000000005</v>
+      </c>
+      <c r="Y6" s="6" cm="1">
+        <f t="array" ref="Y6">IFERROR((X6/W6)*100,NA)</f>
+        <v>98.711757042095343</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -7328,15 +7436,30 @@
         <v>564.05500000000006</v>
       </c>
       <c r="S7" s="6">
-        <f>AVERAGEIFS($J$2:$J$151,$B$2:$B$151,P7)</f>
+        <f t="shared" si="0"/>
         <v>5.8249999999999993</v>
       </c>
-      <c r="T7" s="7">
-        <f>_xlfn.RANK.AVG(S7,$S$2:$S$11,0)</f>
+      <c r="T7" s="1">
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="V7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="W7" s="1" cm="1">
+        <f t="array" ref="W7">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,0,$E$2:$E$151=$V7),0))</f>
+        <v>443.57499999999999</v>
+      </c>
+      <c r="X7" s="1">
+        <f t="array" ref="X7">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,$E$2:$E$151=$V7,0),0))</f>
+        <v>52.28</v>
+      </c>
+      <c r="Y7" s="6" cm="1">
+        <f t="array" ref="Y7">IFERROR((X7/W7)*100,NA)</f>
+        <v>11.786056472975257</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -7385,15 +7508,30 @@
         <v>456.76</v>
       </c>
       <c r="S8" s="6">
-        <f>AVERAGEIFS($J$2:$J$151,$B$2:$B$151,P8)</f>
+        <f t="shared" si="0"/>
         <v>5.6428571428571432</v>
       </c>
-      <c r="T8" s="7">
-        <f>_xlfn.RANK.AVG(S8,$S$2:$S$11,0)</f>
+      <c r="T8" s="1">
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="V8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="W8" s="1" cm="1">
+        <f t="array" ref="W8">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,0,$E$2:$E$151=$V8),0))</f>
+        <v>389.24</v>
+      </c>
+      <c r="X8" s="1">
+        <f t="array" ref="X8">MEDIAN(_xlfn._xlws.FILTER($I$2:$I$151,IF($B$2:$B$151=$P$11,$E$2:$E$151=$V8,0),0))</f>
+        <v>0</v>
+      </c>
+      <c r="Y8" s="6" cm="1">
+        <f t="array" ref="Y8">IFERROR((X8/W8)*100,NA)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -7442,15 +7580,15 @@
         <v>407.91</v>
       </c>
       <c r="S9" s="6">
-        <f>AVERAGEIFS($J$2:$J$151,$B$2:$B$151,P9)</f>
+        <f t="shared" si="0"/>
         <v>5.2533333333333339</v>
       </c>
-      <c r="T9" s="7">
-        <f>_xlfn.RANK.AVG(S9,$S$2:$S$11,0)</f>
+      <c r="T9" s="1">
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -7499,15 +7637,15 @@
         <v>424.72500000000002</v>
       </c>
       <c r="S10" s="6">
-        <f>AVERAGEIFS($J$2:$J$151,$B$2:$B$151,P10)</f>
+        <f t="shared" si="0"/>
         <v>4.6937500000000005</v>
       </c>
-      <c r="T10" s="7">
-        <f>_xlfn.RANK.AVG(S10,$S$2:$S$11,0)</f>
+      <c r="T10" s="1">
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -7556,15 +7694,15 @@
         <v>630.85500000000002</v>
       </c>
       <c r="S11" s="6">
-        <f>AVERAGEIFS($J$2:$J$151,$B$2:$B$151,P11)</f>
+        <f t="shared" si="0"/>
         <v>4.6062500000000002</v>
       </c>
-      <c r="T11" s="7">
-        <f>_xlfn.RANK.AVG(S11,$S$2:$S$11,0)</f>
+      <c r="T11" s="1">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -7602,7 +7740,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -7640,7 +7778,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -7677,8 +7815,17 @@
       <c r="L14" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="P14" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q14" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="R14" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -7715,8 +7862,19 @@
       <c r="L15" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="P15" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q15" s="1">
+        <f>COUNTIFS($C$2:$C$151,P15,$B$2:$B$151,$P$11,$E$2:$E$151,$V$7)</f>
+        <v>0</v>
+      </c>
+      <c r="R15" s="1">
+        <f>SUMIFS($I$2:$I$151,$C$2:$C$151,P15,$B$2:$B$151,$P$11,$E$2:$E$151,$V$7)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -7753,8 +7911,19 @@
       <c r="L16" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="P16" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q16" s="1">
+        <f t="shared" ref="Q16:Q24" si="2">COUNTIFS($C$2:$C$151,P16,$B$2:$B$151,$P$11,$E$2:$E$151,$V$7)</f>
+        <v>0</v>
+      </c>
+      <c r="R16" s="1">
+        <f t="shared" ref="R16:R24" si="3">SUMIFS($I$2:$I$151,$C$2:$C$151,P16,$B$2:$B$151,$P$11,$E$2:$E$151,$V$7)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -7791,8 +7960,19 @@
       <c r="L17" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="P17" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q17" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R17" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -7829,8 +8009,19 @@
       <c r="L18" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="P18" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q18" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R18" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -7867,8 +8058,19 @@
       <c r="L19" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="P19" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q19" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R19" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -7905,8 +8107,19 @@
       <c r="L20" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="P20" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q20" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R20" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -7943,8 +8156,19 @@
       <c r="L21" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="P21" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q21" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R21" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -7981,8 +8205,19 @@
       <c r="L22" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="P22" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q22" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="R22" s="1">
+        <f t="shared" si="3"/>
+        <v>52.28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -8019,8 +8254,19 @@
       <c r="L23" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="P23" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q23" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R23" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -8057,8 +8303,19 @@
       <c r="L24" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="P24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q24" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R24" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -8096,7 +8353,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -8134,7 +8391,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -8172,7 +8429,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -8210,7 +8467,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -8248,7 +8505,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -8286,7 +8543,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -8324,7 +8581,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -12885,23 +13142,20 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="P2:T11">
-    <sortCondition ref="T2:T11"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="P15:P24">
+    <sortCondition ref="P15:P24"/>
   </sortState>
-  <conditionalFormatting sqref="P2:S11">
+  <conditionalFormatting sqref="P2:S11 P14">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>$S2&gt;AVERAGE($S$2:$S$12)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="V1">
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>$S14&gt;AVERAGE($S$2:$S$12)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D99EE96-F80C-404D-963D-ACAA94EBBAE8}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Visualization and Story telling.
</commit_message>
<xml_diff>
--- a/Working/Excel Working/04122025_Winter_Fashion_Trends/Winter_Fashion_Trends_Dataset.xlsx
+++ b/Working/Excel Working/04122025_Winter_Fashion_Trends/Winter_Fashion_Trends_Dataset.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sahil\OneDrive\Documents\Git_Repositories\Daily-Concept-Proofing\Working\Excel Working\04122025_Winter_Fashion_Trends\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6F48B6-E55F-45E9-9D5F-8DE8ABF92BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D203A02-4C00-42B4-9BB9-3401C15EF22D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{4AEEEB2B-2F7C-4B17-B97E-AA8A0F82D82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Winter_Fashion_Trends_DS(OG)" sheetId="1" r:id="rId1"/>
     <sheet name="Analyzing_DS" sheetId="2" r:id="rId2"/>
+    <sheet name="Scatter Plot" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Analyzing_DS!$A$1:$L$151</definedName>
@@ -877,6 +878,1376 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="10"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dPt>
+            <c:idx val="7"/>
+            <c:marker>
+              <c:symbol val="circle"/>
+              <c:size val="10"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:srgbClr val="92D050"/>
+                </a:solidFill>
+                <a:ln w="9525">
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:marker>
+            <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000A-66DD-401D-AD00-4AB166249870}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="9"/>
+            <c:marker>
+              <c:symbol val="circle"/>
+              <c:size val="10"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+                <a:ln w="9525">
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:marker>
+            <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000C-66DD-401D-AD00-4AB166249870}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{94053526-1EAD-44F9-87AC-E6EB937E5760}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-IN"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-66DD-401D-AD00-4AB166249870}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{373F0516-A63D-4571-9507-F91A402C45D4}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-IN"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-66DD-401D-AD00-4AB166249870}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{E911F012-F036-4AF1-B313-76BEA11D5578}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-IN"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-66DD-401D-AD00-4AB166249870}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{B107DE29-734C-4DFA-BCD0-E51C694B1B77}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-IN"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000006-66DD-401D-AD00-4AB166249870}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{CF0DB5A6-E159-432C-9C64-97FF716F15C3}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-IN"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000007-66DD-401D-AD00-4AB166249870}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{4BA6B9A4-4216-46B2-B5D5-9AECDDC618F6}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-IN"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000008-66DD-401D-AD00-4AB166249870}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{6A85B6EC-F3FD-4CF3-9477-AAF12CE1136B}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-IN"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000009-66DD-401D-AD00-4AB166249870}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{F155C390-4A16-4827-BF47-78273EE27790}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-IN"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000A-66DD-401D-AD00-4AB166249870}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="8"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{50727C17-F22D-4A40-973E-DC6F375189AC}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-IN"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000B-66DD-401D-AD00-4AB166249870}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="9"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{A9C93D92-EA06-43C6-8F98-4EAF07A0077F}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-IN"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000C-66DD-401D-AD00-4AB166249870}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showDataLabelsRange val="1"/>
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Analyzing_DS!$Q$2:$Q$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>468.58</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>399.37</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>367.56</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>555.62</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>358.65</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>564.05500000000006</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>456.76</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>407.91</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>424.72500000000002</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>630.85500000000002</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Analyzing_DS!$S$2:$S$11</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.00</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>6.5279999999999996</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6.4846153846153847</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6.4615384615384617</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6.2700000000000005</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5.8549999999999995</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.8249999999999993</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5.6428571428571432</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5.2533333333333339</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4.6937500000000005</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.6062500000000002</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+              <c15:datalabelsRange>
+                <c15:f>Analyzing_DS!$P$2:$P$11</c15:f>
+                <c15:dlblRangeCache>
+                  <c:ptCount val="10"/>
+                  <c:pt idx="0">
+                    <c:v>Mango</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>Zara</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>Nike</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>Adidas</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>North Face</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>Levi's</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>Gucci</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>H&amp;M</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>Prada</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>Uniqlo</c:v>
+                  </c:pt>
+                </c15:dlblRangeCache>
+              </c15:datalabelsRange>
+            </c:ext>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-66DD-401D-AD00-4AB166249870}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1901754816"/>
+        <c:axId val="1901755776"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1901754816"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="300"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1901755776"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1901755776"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="4"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="#,##0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1901754816"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="0.5"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>121920</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>102870</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>594360</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB60309F-C91C-8547-8FFD-56D1A15456AC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -13158,4 +14529,14 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF71541C-336B-42C2-BF4C-CB222824FB68}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>